<commit_message>
Refresh book progress report data
Update the Excel-to-HTML report generator and regenerate the dashboard artifacts for the current book progress snapshot. This includes the latest Excel data, refreshed JSON/HTML output, corrected funnel and stage calculations, and updated pilot labels so the published report matches the latest editorial status.
</commit_message>
<xml_diff>
--- a/book/_static/_reports/progress-2026-09-17.xlsx
+++ b/book/_static/_reports/progress-2026-09-17.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\douden\Documents\GitHub\Calculus\book\_static\_reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C482574E-B785-4C65-9DE1-AD29B3DFD54E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58324EB7-5C5E-423F-B167-FDB2A9A4347D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8370" yWindow="-18870" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11205" yWindow="-21600" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Details" sheetId="1" r:id="rId1"/>
@@ -419,10 +419,10 @@
     <t>A.T. Hensbergen &amp; N.D. Verhulst</t>
   </si>
   <si>
-    <t>EE1G1</t>
-  </si>
-  <si>
-    <t>EE1M2</t>
+    <t>EE1G1 - 2026-2027 Q1</t>
+  </si>
+  <si>
+    <t>EE1M2 - 2026-2027 Q3</t>
   </si>
 </sst>
 </file>
@@ -1342,7 +1342,7 @@
     <col min="8" max="8" width="22.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="I94" s="28"/>
       <c r="J94" s="29"/>
-      <c r="K94" s="12" t="s">
+      <c r="K94" s="3" t="s">
         <v>126</v>
       </c>
       <c r="L94" s="30"/>
@@ -4465,6 +4465,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006787ED29445D224CAD66BC43E8441EB6" ma:contentTypeVersion="4" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="73e358f6993ec21f1771851a5a4960ab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7ddafb96-d811-4186-8639-85d6b875f2ea" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="536da21993cd937d3c98c599ab6065f2" ns2:_="">
     <xsd:import namespace="7ddafb96-d811-4186-8639-85d6b875f2ea"/>
@@ -4608,12 +4614,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79EC5FC4-DC1C-4FCF-AE42-23EB7ED0542E}">
   <ds:schemaRefs>
@@ -4623,6 +4623,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{280A695D-2E37-4619-B5DA-381BDBA7B958}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62AA9F17-6CF4-427B-A981-E944979DE167}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4638,13 +4647,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{280A695D-2E37-4619-B5DA-381BDBA7B958}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>